<commit_message>
intégration du mode kiosque
et fix du junk drop rate.
et nouveau tuning de la difficulté.
</commit_message>
<xml_diff>
--- a/DifficultyProgression.xlsx
+++ b/DifficultyProgression.xlsx
@@ -5,15 +5,16 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GITHUB\DiceRoyal\Mobile\datafiles\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GITHUB\DiceRoyal\Mobile\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4B7AB25-FC8C-4581-858F-9C27FCAF899F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B198589E-72D3-4C3B-BA0B-3C2C8D834183}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{5FC277F8-3D03-4D3F-9864-CF296E7B8EB1}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{5FC277F8-3D03-4D3F-9864-CF296E7B8EB1}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -644,13 +645,13 @@
         <v>13</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="I3" s="1" t="s">
         <v>13</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="K3" s="1" t="s">
         <v>13</v>
@@ -677,15 +678,15 @@
       <c r="G4" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="H4" s="1"/>
+      <c r="H4" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="I4" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="J4" s="1"/>
+      <c r="K4" s="1" t="s">
         <v>14</v>
-      </c>
-      <c r="J4" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="K4" s="1" t="s">
-        <v>13</v>
       </c>
       <c r="L4" s="1" t="s">
         <v>20</v>
@@ -711,14 +712,13 @@
       <c r="G5" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="H5" s="1"/>
-      <c r="I5" s="1"/>
-      <c r="J5" s="1" t="s">
+      <c r="H5" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="I5" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="K5" s="1" t="s">
-        <v>13</v>
-      </c>
+      <c r="K5" s="1"/>
       <c r="L5" s="1" t="s">
         <v>21</v>
       </c>
@@ -743,12 +743,11 @@
       <c r="G6" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="H6" s="1"/>
+      <c r="H6" s="1" t="s">
+        <v>16</v>
+      </c>
       <c r="I6" s="1"/>
       <c r="J6" s="1"/>
-      <c r="K6" s="1" t="s">
-        <v>14</v>
-      </c>
       <c r="L6" s="1" t="s">
         <v>22</v>
       </c>
@@ -1125,4 +1124,268 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{192050DF-0539-4C68-A6C8-F41BFCC373FF}">
+  <dimension ref="L1:P20"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="12:16" x14ac:dyDescent="0.25">
+      <c r="L1">
+        <v>0</v>
+      </c>
+      <c r="P1">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="2" spans="12:16" x14ac:dyDescent="0.25">
+      <c r="L2">
+        <f>SUM(L1+M2)</f>
+        <v>5000</v>
+      </c>
+      <c r="M2">
+        <v>5000</v>
+      </c>
+      <c r="P2">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="3" spans="12:16" x14ac:dyDescent="0.25">
+      <c r="L3">
+        <f t="shared" ref="L3:L20" si="0">SUM(L2+M3)</f>
+        <v>15000</v>
+      </c>
+      <c r="M3">
+        <f>SUM(M2+5000)</f>
+        <v>10000</v>
+      </c>
+      <c r="P3">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="4" spans="12:16" x14ac:dyDescent="0.25">
+      <c r="L4">
+        <f t="shared" si="0"/>
+        <v>30000</v>
+      </c>
+      <c r="M4">
+        <f t="shared" ref="M4:M20" si="1">SUM(M3+5000)</f>
+        <v>15000</v>
+      </c>
+      <c r="P4">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="5" spans="12:16" x14ac:dyDescent="0.25">
+      <c r="L5">
+        <f t="shared" si="0"/>
+        <v>50000</v>
+      </c>
+      <c r="M5">
+        <f t="shared" si="1"/>
+        <v>20000</v>
+      </c>
+      <c r="P5">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="6" spans="12:16" x14ac:dyDescent="0.25">
+      <c r="L6">
+        <f t="shared" si="0"/>
+        <v>75000</v>
+      </c>
+      <c r="M6">
+        <f t="shared" si="1"/>
+        <v>25000</v>
+      </c>
+      <c r="P6">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="7" spans="12:16" x14ac:dyDescent="0.25">
+      <c r="L7">
+        <f t="shared" si="0"/>
+        <v>105000</v>
+      </c>
+      <c r="M7">
+        <f t="shared" si="1"/>
+        <v>30000</v>
+      </c>
+      <c r="P7">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="8" spans="12:16" x14ac:dyDescent="0.25">
+      <c r="L8">
+        <f t="shared" si="0"/>
+        <v>140000</v>
+      </c>
+      <c r="M8">
+        <f t="shared" si="1"/>
+        <v>35000</v>
+      </c>
+      <c r="P8">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="9" spans="12:16" x14ac:dyDescent="0.25">
+      <c r="L9">
+        <f t="shared" si="0"/>
+        <v>180000</v>
+      </c>
+      <c r="M9">
+        <f t="shared" si="1"/>
+        <v>40000</v>
+      </c>
+      <c r="P9">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="10" spans="12:16" x14ac:dyDescent="0.25">
+      <c r="L10">
+        <f t="shared" si="0"/>
+        <v>225000</v>
+      </c>
+      <c r="M10">
+        <f t="shared" si="1"/>
+        <v>45000</v>
+      </c>
+      <c r="P10">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="11" spans="12:16" x14ac:dyDescent="0.25">
+      <c r="L11">
+        <f t="shared" si="0"/>
+        <v>275000</v>
+      </c>
+      <c r="M11">
+        <f t="shared" si="1"/>
+        <v>50000</v>
+      </c>
+      <c r="P11">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="12" spans="12:16" x14ac:dyDescent="0.25">
+      <c r="L12">
+        <f t="shared" si="0"/>
+        <v>330000</v>
+      </c>
+      <c r="M12">
+        <f t="shared" si="1"/>
+        <v>55000</v>
+      </c>
+      <c r="P12">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="13" spans="12:16" x14ac:dyDescent="0.25">
+      <c r="L13">
+        <f t="shared" si="0"/>
+        <v>390000</v>
+      </c>
+      <c r="M13">
+        <f t="shared" si="1"/>
+        <v>60000</v>
+      </c>
+      <c r="P13">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="14" spans="12:16" x14ac:dyDescent="0.25">
+      <c r="L14">
+        <f t="shared" si="0"/>
+        <v>455000</v>
+      </c>
+      <c r="M14">
+        <f t="shared" si="1"/>
+        <v>65000</v>
+      </c>
+      <c r="P14">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="15" spans="12:16" x14ac:dyDescent="0.25">
+      <c r="L15">
+        <f t="shared" si="0"/>
+        <v>525000</v>
+      </c>
+      <c r="M15">
+        <f t="shared" si="1"/>
+        <v>70000</v>
+      </c>
+      <c r="P15">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="16" spans="12:16" x14ac:dyDescent="0.25">
+      <c r="L16">
+        <f t="shared" si="0"/>
+        <v>600000</v>
+      </c>
+      <c r="M16">
+        <f t="shared" si="1"/>
+        <v>75000</v>
+      </c>
+      <c r="P16">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="17" spans="12:16" x14ac:dyDescent="0.25">
+      <c r="L17">
+        <f t="shared" si="0"/>
+        <v>680000</v>
+      </c>
+      <c r="M17">
+        <f t="shared" si="1"/>
+        <v>80000</v>
+      </c>
+      <c r="P17">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="18" spans="12:16" x14ac:dyDescent="0.25">
+      <c r="L18">
+        <f t="shared" si="0"/>
+        <v>765000</v>
+      </c>
+      <c r="M18">
+        <f t="shared" si="1"/>
+        <v>85000</v>
+      </c>
+      <c r="P18">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="19" spans="12:16" x14ac:dyDescent="0.25">
+      <c r="L19">
+        <f t="shared" si="0"/>
+        <v>855000</v>
+      </c>
+      <c r="M19">
+        <f t="shared" si="1"/>
+        <v>90000</v>
+      </c>
+      <c r="P19">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="20" spans="12:16" x14ac:dyDescent="0.25">
+      <c r="L20">
+        <f t="shared" si="0"/>
+        <v>950000</v>
+      </c>
+      <c r="M20">
+        <f t="shared" si="1"/>
+        <v>95000</v>
+      </c>
+      <c r="P20">
+        <v>0.1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>